<commit_message>
Load anchor towns from geo lookup
Move anchor-town configuration into pipeline/geo/geo_lookup.xlsx, validate required mappings, and preserve the existing six live-slice outputs.
</commit_message>
<xml_diff>
--- a/pipeline/geo/geo_lookup.xlsx
+++ b/pipeline/geo/geo_lookup.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re96aaac029b64122"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_log" sheetId="2" r:id="Rd42abc8068534aaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_required" sheetId="3" r:id="R90262d90ef254bbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster_summary" sheetId="4" r:id="Rd7d3c86d8c2e4ced"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_me" sheetId="5" r:id="R02cb610123f54781"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LocationFallback" sheetId="6" r:id="R8924ad9c4ef24407"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6019ff021b204a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_log" sheetId="2" r:id="Rbd693daeb3484ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_required" sheetId="3" r:id="R06676a6ed9d849e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster_summary" sheetId="4" r:id="Rcf6e15a611e5409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_me" sheetId="5" r:id="Rb76295698fd14342"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LocationFallback" sheetId="6" r:id="R32cd1a989e664f6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anchor_towns" sheetId="7" r:id="R71bb3017941e4eb8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3169,7 +3170,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3196,6 +3197,11 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -3205,7 +3211,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -3289,6 +3295,17 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3362,6 +3379,17 @@
     <x:tableColumn id="2" name="Cluster"/>
     <x:tableColumn id="3" name="Status"/>
     <x:tableColumn id="4" name="Notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="AnchorTownsTable" displayName="AnchorTownsTable" ref="A1:C7" headerRowCount="1">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="region"/>
+    <x:tableColumn id="2" name="category"/>
+    <x:tableColumn id="3" name="anchor_town"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
@@ -13115,7 +13143,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff378e6d2c664b7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b6af130e4104078"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27812,7 +27840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b0b9a95884d4946"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9fdf3ced37b4337"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30049,7 +30077,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7620f2152f54e95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf178d0c17244d1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30854,7 +30882,106 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racdddd07e2bf4fed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4baf9075d4004f4b"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="39" t="str">
+        <x:v>region</x:v>
+      </x:c>
+      <x:c r="B1" s="39" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="C1" s="39" t="str">
+        <x:v>anchor_town</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="22" t="str">
+        <x:v>West Yorkshire</x:v>
+      </x:c>
+      <x:c r="B2" s="22" t="str">
+        <x:v>admin_service</x:v>
+      </x:c>
+      <x:c r="C2" s="22" t="str">
+        <x:v>Leeds</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="22" t="str">
+        <x:v>South Yorkshire</x:v>
+      </x:c>
+      <x:c r="B3" s="22" t="str">
+        <x:v>admin_service</x:v>
+      </x:c>
+      <x:c r="C3" s="22" t="str">
+        <x:v>Sheffield</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="22" t="str">
+        <x:v>North East</x:v>
+      </x:c>
+      <x:c r="B4" s="22" t="str">
+        <x:v>admin_service</x:v>
+      </x:c>
+      <x:c r="C4" s="22" t="str">
+        <x:v>Newcastle Upon Tyne</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="22" t="str">
+        <x:v>West Yorkshire</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>support_worker</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>Leeds</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="22" t="str">
+        <x:v>South Yorkshire</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>support_worker</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>Sheffield</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="22" t="str">
+        <x:v>North East</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>support_worker</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>Newcastle Upon Tyne</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="B2:B100">
+      <x:formula1>"admin_service,support_worker"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0722c8bf8844f5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Standardise Yorkshire region identifiers
Standardise production and geo lookup identifiers to Yorkshire - West and Yorkshire - South while preserving existing public routes, output filenames, and six-slice production behaviour.
</commit_message>
<xml_diff>
--- a/pipeline/geo/geo_lookup.xlsx
+++ b/pipeline/geo/geo_lookup.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6019ff021b204a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_log" sheetId="2" r:id="Rbd693daeb3484ca8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_required" sheetId="3" r:id="R06676a6ed9d849e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster_summary" sheetId="4" r:id="Rcf6e15a611e5409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_me" sheetId="5" r:id="Rb76295698fd14342"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LocationFallback" sheetId="6" r:id="R32cd1a989e664f6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anchor_towns" sheetId="7" r:id="R71bb3017941e4eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R092f7fe2c229434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change_log" sheetId="2" r:id="Rfb87fd931d154bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_required" sheetId="3" r:id="Rd6daf09e4a724580"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cluster_summary" sheetId="4" r:id="R5533e69880a74a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_me" sheetId="5" r:id="R1ec60975476442a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LocationFallback" sheetId="6" r:id="R47bf14c7734e4c99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anchor_towns" sheetId="7" r:id="R733a4ca80b3c43d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13143,7 +13143,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b6af130e4104078"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R619e7a883a30473e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27840,7 +27840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9fdf3ced37b4337"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85f7cb209b174227"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30077,7 +30077,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf178d0c17244d1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32bfc0ac2a99462a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30882,7 +30882,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4baf9075d4004f4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redb1a37f7d3b4935"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30909,7 +30909,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="22" t="str">
-        <x:v>West Yorkshire</x:v>
+        <x:v>Yorkshire - West</x:v>
       </x:c>
       <x:c r="B2" s="22" t="str">
         <x:v>admin_service</x:v>
@@ -30920,7 +30920,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="22" t="str">
-        <x:v>South Yorkshire</x:v>
+        <x:v>Yorkshire - South</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
         <x:v>admin_service</x:v>
@@ -30942,7 +30942,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="22" t="str">
-        <x:v>West Yorkshire</x:v>
+        <x:v>Yorkshire - West</x:v>
       </x:c>
       <x:c r="B5" s="22" t="str">
         <x:v>support_worker</x:v>
@@ -30953,7 +30953,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="22" t="str">
-        <x:v>South Yorkshire</x:v>
+        <x:v>Yorkshire - South</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
         <x:v>support_worker</x:v>
@@ -30981,7 +30981,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0722c8bf8844f5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c35b3422d4346c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Build Cumbria South support-worker production slice
</commit_message>
<xml_diff>
--- a/pipeline/geo/geo_lookup.xlsx
+++ b/pipeline/geo/geo_lookup.xlsx
@@ -41921,7 +41921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -42096,6 +42096,23 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>Southampton</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cumbria - South</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>support_worker</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Barrow-in-Furness</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix canonical Legal geo gaps
</commit_message>
<xml_diff>
--- a/pipeline/geo/geo_lookup.xlsx
+++ b/pipeline/geo/geo_lookup.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1207"/>
+  <dimension ref="A1:B1208"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>East of England</t>
+          <t>Norfolk</t>
         </is>
       </c>
     </row>
@@ -14915,6 +14915,18 @@
       <c r="B1207" t="inlineStr">
         <is>
           <t>West Midlands - Birmingham &amp; Solihull</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>Studley</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>West Midlands - Coventry &amp; Warwickshire</t>
         </is>
       </c>
     </row>
@@ -40870,7 +40882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -41998,6 +42010,60 @@
           <t>AUTO</t>
         </is>
       </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Sheffield</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Yorkshire - South</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Leeds</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Yorkshire - West</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Belfast</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Northern Ireland - East</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C51">

</xml_diff>